<commit_message>
Add Copyright and Version
Update BRD Version
Added Footer to the Spreadsheet
</commit_message>
<xml_diff>
--- a/NeuByteTechnologies/FitnessApp/docs/RTM/NeuByteFitnessAppRequirementTracabilityMatrix.xlsx
+++ b/NeuByteTechnologies/FitnessApp/docs/RTM/NeuByteFitnessAppRequirementTracabilityMatrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\portfolio\NeuByteTechnologies\FitnessApp\docs\RTM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DA58F36C-E696-4047-B457-DEB76F195FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACA159B-586A-4650-A23E-FC72BA0DDB91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{F206755B-748C-4243-AFE7-269C66BA7D5C}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F206755B-748C-4243-AFE7-269C66BA7D5C}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginRTM" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Sheet1!$A$1:$A$385</definedName>
   </definedNames>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -23078,8 +23077,11 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N267">
     <sortCondition ref="A2:A267"/>
   </sortState>
-  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="3" scale="57" fitToHeight="0" orientation="landscape" horizontalDpi="4294967293" r:id="rId1"/>
+  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.75" header="0.3" footer="0.5"/>
+  <pageSetup paperSize="3" scale="42" fitToHeight="0" orientation="landscape" horizontalDpi="4294967293" r:id="rId1"/>
+  <headerFooter scaleWithDoc="0">
+    <oddFooter>&amp;L© 2026 NeuByte Technologies, All Rights Reserved – Version: 1.0</oddFooter>
+  </headerFooter>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
version favicon to kill cache
</commit_message>
<xml_diff>
--- a/NeuByteTechnologies/FitnessApp/docs/RTM/NeuByteFitnessAppRequirementTracabilityMatrix.xlsx
+++ b/NeuByteTechnologies/FitnessApp/docs/RTM/NeuByteFitnessAppRequirementTracabilityMatrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\portfolio\NeuByteTechnologies\FitnessApp\docs\RTM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACA159B-586A-4650-A23E-FC72BA0DDB91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB32AC50-CCDF-4FC4-849D-BA4A4BB53AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F206755B-748C-4243-AFE7-269C66BA7D5C}"/>
   </bookViews>
@@ -23077,10 +23077,11 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N267">
     <sortCondition ref="A2:A267"/>
   </sortState>
-  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.75" header="0.3" footer="0.5"/>
-  <pageSetup paperSize="3" scale="42" fitToHeight="0" orientation="landscape" horizontalDpi="4294967293" r:id="rId1"/>
+  <printOptions headings="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="3" scale="41" fitToHeight="0" orientation="landscape" horizontalDpi="4294967293" r:id="rId1"/>
   <headerFooter scaleWithDoc="0">
-    <oddFooter>&amp;L© 2026 NeuByte Technologies, All Rights Reserved – Version: 1.0</oddFooter>
+    <oddFooter>&amp;L© 2026 NeuByte Technologies, All Rights Reserved&amp;RVersion: 1.0</oddFooter>
   </headerFooter>
 </worksheet>
 </file>

</xml_diff>